<commit_message>
version 08 - Add child component to handling component easily
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Website_NenThomBnC\Website_NenThomBnC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0911C529-D878-4D4C-A74C-6E0FB72B437C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E81537-904F-4BFE-A0D9-8F7CFE7BA982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3DCBFBA-82F4-4982-9C95-CC18301E2A03}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E3DCBFBA-82F4-4982-9C95-CC18301E2A03}"/>
   </bookViews>
   <sheets>
     <sheet name="Before" sheetId="1" r:id="rId1"/>
     <sheet name="After" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1116,6 +1115,24 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1133,24 +1150,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1515,26 +1514,26 @@
       </c>
     </row>
     <row r="2" spans="2:8" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="39"/>
-      <c r="E2" s="38" t="s">
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="42" t="s">
+      <c r="F2" s="33"/>
+      <c r="G2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="36" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="2" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="41"/>
+      <c r="B3" s="35"/>
       <c r="C3" s="22" t="s">
         <v>53</v>
       </c>
@@ -1547,11 +1546,11 @@
       <c r="F3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
     </row>
     <row r="4" spans="2:8" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="40" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -1569,12 +1568,12 @@
       <c r="G4" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="H4" s="42" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="35"/>
+      <c r="B5" s="41"/>
       <c r="C5" s="8" t="s">
         <v>52</v>
       </c>
@@ -1587,8 +1586,8 @@
       <c r="F5" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
@@ -1781,7 +1780,7 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="38" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1800,7 +1799,7 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="32"/>
+      <c r="B17" s="38"/>
       <c r="C17" s="8" t="s">
         <v>42</v>
       </c>
@@ -1813,7 +1812,7 @@
       <c r="H17" s="46"/>
     </row>
     <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="32"/>
+      <c r="B18" s="38"/>
       <c r="C18" s="8" t="s">
         <v>43</v>
       </c>
@@ -1826,7 +1825,7 @@
       <c r="H18" s="46"/>
     </row>
     <row r="19" spans="2:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32"/>
+      <c r="B19" s="38"/>
       <c r="C19" s="8" t="s">
         <v>44</v>
       </c>
@@ -1839,7 +1838,7 @@
       <c r="H19" s="46"/>
     </row>
     <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="38" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="47" t="s">
@@ -1853,12 +1852,12 @@
       <c r="G20" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="33" t="s">
+      <c r="H20" s="39" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="32"/>
+      <c r="B21" s="38"/>
       <c r="C21" s="47"/>
       <c r="D21" s="4"/>
       <c r="E21" s="8" t="s">
@@ -1869,7 +1868,7 @@
       <c r="H21" s="31"/>
     </row>
     <row r="22" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="38" t="s">
         <v>28</v>
       </c>
       <c r="C22" s="47" t="s">
@@ -1883,12 +1882,12 @@
       <c r="G22" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H22" s="33" t="s">
+      <c r="H22" s="39" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32"/>
+      <c r="B23" s="38"/>
       <c r="C23" s="47"/>
       <c r="D23" s="4"/>
       <c r="E23" s="8" t="s">
@@ -1918,7 +1917,7 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="142.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="38" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -1932,12 +1931,12 @@
       <c r="G25" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H25" s="33" t="s">
+      <c r="H25" s="39" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="258.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="32"/>
+      <c r="B26" s="38"/>
       <c r="C26" s="8" t="s">
         <v>50</v>
       </c>
@@ -1989,12 +1988,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G2:G3"/>
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="G25:G26"/>
     <mergeCell ref="B25:B26"/>
@@ -2011,6 +2004,12 @@
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="H22:H23"/>
     <mergeCell ref="G16:G19"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2036,26 +2035,26 @@
       </c>
     </row>
     <row r="2" spans="2:8" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="39"/>
-      <c r="E2" s="38" t="s">
+      <c r="D2" s="33"/>
+      <c r="E2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="42" t="s">
+      <c r="F2" s="33"/>
+      <c r="G2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="H2" s="36" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="2" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="41"/>
+      <c r="B3" s="35"/>
       <c r="C3" s="22" t="s">
         <v>53</v>
       </c>
@@ -2068,11 +2067,11 @@
       <c r="F3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
     </row>
     <row r="4" spans="2:8" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="40" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -2090,12 +2089,12 @@
       <c r="G4" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="36" t="s">
+      <c r="H4" s="42" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="35"/>
+      <c r="B5" s="41"/>
       <c r="C5" s="8" t="s">
         <v>52</v>
       </c>
@@ -2108,16 +2107,15 @@
       <c r="F5" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="7"/>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="28"/>
+      <c r="E6" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="5"/>
       <c r="F6" s="27"/>
       <c r="G6" s="9"/>
       <c r="H6" s="9"/>
@@ -2313,7 +2311,7 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="38" t="s">
         <v>24</v>
       </c>
       <c r="C17" s="8" t="s">
@@ -2332,7 +2330,7 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="32"/>
+      <c r="B18" s="38"/>
       <c r="C18" s="8" t="s">
         <v>42</v>
       </c>
@@ -2345,7 +2343,7 @@
       <c r="H18" s="46"/>
     </row>
     <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="32"/>
+      <c r="B19" s="38"/>
       <c r="C19" s="8" t="s">
         <v>43</v>
       </c>
@@ -2358,7 +2356,7 @@
       <c r="H19" s="46"/>
     </row>
     <row r="20" spans="2:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="32"/>
+      <c r="B20" s="38"/>
       <c r="C20" s="8" t="s">
         <v>44</v>
       </c>
@@ -2371,7 +2369,7 @@
       <c r="H20" s="46"/>
     </row>
     <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="38" t="s">
         <v>26</v>
       </c>
       <c r="C21" s="47" t="s">
@@ -2385,12 +2383,12 @@
       <c r="G21" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="H21" s="33" t="s">
+      <c r="H21" s="39" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="32"/>
+      <c r="B22" s="38"/>
       <c r="C22" s="47"/>
       <c r="D22" s="4"/>
       <c r="E22" s="8" t="s">
@@ -2401,7 +2399,7 @@
       <c r="H22" s="31"/>
     </row>
     <row r="23" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="38" t="s">
         <v>28</v>
       </c>
       <c r="C23" s="47" t="s">
@@ -2415,12 +2413,12 @@
       <c r="G23" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H23" s="33" t="s">
+      <c r="H23" s="39" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="32"/>
+      <c r="B24" s="38"/>
       <c r="C24" s="47"/>
       <c r="D24" s="4"/>
       <c r="E24" s="8" t="s">
@@ -2450,7 +2448,7 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="142.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="38" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="8" t="s">
@@ -2464,12 +2462,12 @@
       <c r="G26" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="33" t="s">
+      <c r="H26" s="39" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="258.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="32"/>
+      <c r="B27" s="38"/>
       <c r="C27" s="8" t="s">
         <v>50</v>
       </c>
@@ -2521,6 +2519,21 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="G17:G20"/>
+    <mergeCell ref="H17:H20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="G23:G24"/>
@@ -2528,21 +2541,6 @@
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="G26:G27"/>
     <mergeCell ref="H26:H27"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="G17:G20"/>
-    <mergeCell ref="H17:H20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
version 11 - Improve product filter by search and add detail information component and initial payment version page
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Website_NenThomBnC\Website_NenThomBnC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E81537-904F-4BFE-A0D9-8F7CFE7BA982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C22F977-564A-4534-B58D-901AC17C67B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E3DCBFBA-82F4-4982-9C95-CC18301E2A03}"/>
   </bookViews>
@@ -724,7 +724,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -743,6 +743,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -1022,7 +1028,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1115,6 +1121,36 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1133,35 +1169,11 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1514,26 +1526,26 @@
       </c>
     </row>
     <row r="2" spans="2:8" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="D2" s="43"/>
+      <c r="E2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="36" t="s">
+      <c r="F2" s="43"/>
+      <c r="G2" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="36" t="s">
+      <c r="H2" s="46" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="2" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="35"/>
+      <c r="B3" s="45"/>
       <c r="C3" s="22" t="s">
         <v>53</v>
       </c>
@@ -1546,11 +1558,11 @@
       <c r="F3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
     </row>
     <row r="4" spans="2:8" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="34" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -1565,15 +1577,15 @@
       <c r="F4" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="42" t="s">
+      <c r="H4" s="36" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="41"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="8" t="s">
         <v>52</v>
       </c>
@@ -1586,8 +1598,8 @@
       <c r="F5" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
@@ -1780,7 +1792,7 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="32" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -1791,15 +1803,15 @@
         <v>6</v>
       </c>
       <c r="F16" s="18"/>
-      <c r="G16" s="46" t="s">
+      <c r="G16" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="H16" s="45" t="s">
+      <c r="H16" s="39" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="38"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="8" t="s">
         <v>42</v>
       </c>
@@ -1808,11 +1820,11 @@
         <v>6</v>
       </c>
       <c r="F17" s="18"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="46"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
     </row>
     <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="38"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="8" t="s">
         <v>43</v>
       </c>
@@ -1821,11 +1833,11 @@
         <v>6</v>
       </c>
       <c r="F18" s="18"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
     </row>
     <row r="19" spans="2:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="38"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="8" t="s">
         <v>44</v>
       </c>
@@ -1834,14 +1846,14 @@
         <v>6</v>
       </c>
       <c r="F19" s="18"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="46"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
     </row>
     <row r="20" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="47" t="s">
+      <c r="C20" s="41" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="4"/>
@@ -1852,13 +1864,13 @@
       <c r="G20" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="H20" s="39" t="s">
+      <c r="H20" s="33" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="38"/>
-      <c r="C21" s="47"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="4"/>
       <c r="E21" s="8" t="s">
         <v>47</v>
@@ -1868,10 +1880,10 @@
       <c r="H21" s="31"/>
     </row>
     <row r="22" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="47" t="s">
+      <c r="C22" s="41" t="s">
         <v>38</v>
       </c>
       <c r="D22" s="4"/>
@@ -1882,13 +1894,13 @@
       <c r="G22" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H22" s="39" t="s">
+      <c r="H22" s="33" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="38"/>
-      <c r="C23" s="47"/>
+      <c r="B23" s="32"/>
+      <c r="C23" s="41"/>
       <c r="D23" s="4"/>
       <c r="E23" s="8" t="s">
         <v>49</v>
@@ -1917,7 +1929,7 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="142.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="38" t="s">
+      <c r="B25" s="32" t="s">
         <v>32</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -1931,12 +1943,12 @@
       <c r="G25" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H25" s="39" t="s">
+      <c r="H25" s="33" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="258.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="38"/>
+      <c r="B26" s="32"/>
       <c r="C26" s="8" t="s">
         <v>50</v>
       </c>
@@ -1988,6 +2000,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="G2:G3"/>
     <mergeCell ref="G22:G23"/>
     <mergeCell ref="G25:G26"/>
     <mergeCell ref="B25:B26"/>
@@ -2004,12 +2022,6 @@
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="H22:H23"/>
     <mergeCell ref="G16:G19"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2035,26 +2047,26 @@
       </c>
     </row>
     <row r="2" spans="2:8" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="33"/>
-      <c r="E2" s="32" t="s">
+      <c r="D2" s="43"/>
+      <c r="E2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="36" t="s">
+      <c r="F2" s="43"/>
+      <c r="G2" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="36" t="s">
+      <c r="H2" s="46" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="2:8" s="2" customFormat="1" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="35"/>
+      <c r="B3" s="45"/>
       <c r="C3" s="22" t="s">
         <v>53</v>
       </c>
@@ -2067,11 +2079,11 @@
       <c r="F3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
     </row>
     <row r="4" spans="2:8" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="34" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -2086,15 +2098,15 @@
       <c r="F4" s="26" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="42" t="s">
+      <c r="H4" s="36" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="41"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="8" t="s">
         <v>52</v>
       </c>
@@ -2107,8 +2119,8 @@
       <c r="F5" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="2:8" s="2" customFormat="1" ht="176.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="7"/>
@@ -2311,7 +2323,7 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="32" t="s">
         <v>24</v>
       </c>
       <c r="C17" s="8" t="s">
@@ -2322,15 +2334,15 @@
         <v>6</v>
       </c>
       <c r="F17" s="18"/>
-      <c r="G17" s="46" t="s">
+      <c r="G17" s="40" t="s">
         <v>25</v>
       </c>
-      <c r="H17" s="45" t="s">
+      <c r="H17" s="39" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B18" s="38"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="8" t="s">
         <v>42</v>
       </c>
@@ -2339,11 +2351,11 @@
         <v>6</v>
       </c>
       <c r="F18" s="18"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="46"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
     </row>
     <row r="19" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B19" s="38"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="8" t="s">
         <v>43</v>
       </c>
@@ -2352,11 +2364,11 @@
         <v>6</v>
       </c>
       <c r="F19" s="18"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="46"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="40"/>
     </row>
     <row r="20" spans="2:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="38"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="8" t="s">
         <v>44</v>
       </c>
@@ -2365,14 +2377,14 @@
         <v>6</v>
       </c>
       <c r="F20" s="18"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="40"/>
     </row>
     <row r="21" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="47" t="s">
+      <c r="C21" s="41" t="s">
         <v>45</v>
       </c>
       <c r="D21" s="4"/>
@@ -2383,13 +2395,13 @@
       <c r="G21" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="H21" s="39" t="s">
+      <c r="H21" s="33" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="38"/>
-      <c r="C22" s="47"/>
+      <c r="B22" s="32"/>
+      <c r="C22" s="41"/>
       <c r="D22" s="4"/>
       <c r="E22" s="8" t="s">
         <v>47</v>
@@ -2399,10 +2411,10 @@
       <c r="H22" s="31"/>
     </row>
     <row r="23" spans="2:8" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="38" t="s">
+      <c r="B23" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="47" t="s">
+      <c r="C23" s="41" t="s">
         <v>38</v>
       </c>
       <c r="D23" s="4"/>
@@ -2413,13 +2425,13 @@
       <c r="G23" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="H23" s="39" t="s">
+      <c r="H23" s="33" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="38"/>
-      <c r="C24" s="47"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="41"/>
       <c r="D24" s="4"/>
       <c r="E24" s="8" t="s">
         <v>49</v>
@@ -2448,10 +2460,10 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="142.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="48" t="s">
         <v>38</v>
       </c>
       <c r="D26" s="8"/>
@@ -2462,17 +2474,17 @@
       <c r="G26" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="H26" s="39" t="s">
+      <c r="H26" s="33" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="258.60000000000002" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="38"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="8" t="s">
         <v>50</v>
       </c>
       <c r="D27" s="8"/>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="49" t="s">
         <v>51</v>
       </c>
       <c r="F27" s="20"/>
@@ -2519,6 +2531,20 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="G17:G20"/>
+    <mergeCell ref="H17:H20"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="G4:G5"/>
     <mergeCell ref="H4:H5"/>
@@ -2527,20 +2553,6 @@
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="H2:H3"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="G17:G20"/>
-    <mergeCell ref="H17:H20"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H26:H27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
version 19 - Improve Another_information component
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -29,8 +29,154 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>PC</author>
+  </authors>
+  <commentList>
+    <comment ref="K16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Buld later</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K17" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Buld later
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K18" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Handle internal in Angular, dont contact to server now</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Handle internal in Angular, dont contact to server now
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K20" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Handle internal in Angular, dont contact to server now
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K21" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Handle internal in Angular, dont contact to server now
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="151">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -154,6 +300,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">- Read user information from Session storage (Redis in this case), next 2 steps:
 + If have data (defined user) </t>
     </r>
@@ -329,6 +480,9 @@
     <t>/api/news</t>
   </si>
   <si>
+    <t>Not Applicable seperatedly for now. Build later</t>
+  </si>
+  <si>
     <t>NEWS_URL</t>
   </si>
   <si>
@@ -469,6 +623,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -529,6 +689,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>+ If user is added sucessully:</t>
     </r>
     <r>
@@ -584,6 +750,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -713,6 +885,31 @@
   <si>
     <t>SHOPPING_BAG_HANDLING_URL</t>
   </si>
+  <si>
+    <t>API 19: Serve Angular app</t>
+  </si>
+  <si>
+    <t>public/dist/index.html</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> *</t>
+  </si>
+  <si>
+    <t>Serve all Angular static file after build for production.
+Combined Angular static files and Express server followed with Modular Monolith architecture</t>
+  </si>
+  <si>
+    <t>All route request of Internal Angular (not API call of Server)</t>
+  </si>
+  <si>
+    <t>index.html of corresponding Angular route</t>
+  </si>
+  <si>
+    <t>All internal Angular routing</t>
+  </si>
 </sst>
 </file>
 
@@ -767,12 +964,6 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
@@ -794,13 +985,6 @@
       <sz val="12"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -951,6 +1135,17 @@
       <name val="Arial"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
   </fonts>
   <fills count="40">
     <fill>
@@ -997,7 +1192,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.5"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1312,19 +1507,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1333,131 +1537,122 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1465,14 +1660,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1484,12 +1673,12 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1499,113 +1688,95 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -1953,799 +2124,830 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
-    <col min="1" max="1" width="38.5833333333333" style="3" customWidth="1"/>
-    <col min="2" max="2" width="33.5277777777778" style="3" customWidth="1"/>
-    <col min="3" max="3" width="31.4259259259259" style="3" customWidth="1"/>
-    <col min="4" max="4" width="51.3055555555556" style="4" customWidth="1"/>
-    <col min="5" max="5" width="72.8055555555556" style="5" customWidth="1"/>
-    <col min="6" max="6" width="51.4259259259259" style="3" customWidth="1"/>
-    <col min="7" max="7" width="92.6944444444444" style="3" customWidth="1"/>
-    <col min="8" max="8" width="74.7407407407407" style="5" customWidth="1"/>
-    <col min="9" max="9" width="56.6574074074074" style="3" customWidth="1"/>
-    <col min="10" max="10" width="89.8333333333333" style="3" customWidth="1"/>
-    <col min="11" max="11" width="66.4444444444444" style="3" customWidth="1"/>
-    <col min="12" max="16384" width="9" style="6"/>
+    <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.525" style="2" customWidth="1"/>
+    <col min="3" max="3" width="31.425" style="2" customWidth="1"/>
+    <col min="4" max="4" width="51.3083333333333" style="3" customWidth="1"/>
+    <col min="5" max="5" width="72.8083333333333" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.425" style="2" customWidth="1"/>
+    <col min="7" max="7" width="92.6916666666667" style="2" customWidth="1"/>
+    <col min="8" max="8" width="74.7416666666667" style="1" customWidth="1"/>
+    <col min="9" max="9" width="56.6583333333333" style="2" customWidth="1"/>
+    <col min="10" max="10" width="89.8333333333333" style="2" customWidth="1"/>
+    <col min="11" max="11" width="66.4416666666667" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.8" spans="1:1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="1" ht="27.6" customHeight="1" spans="1:11">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="14" t="s">
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="39" t="s">
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="34" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" ht="35.4" customHeight="1" spans="1:11">
-      <c r="A3" s="15"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="17" t="s">
+      <c r="A3" s="6"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="17" t="s">
+      <c r="G3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="40"/>
+      <c r="K3" s="35"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="47" t="s">
+      <c r="G4" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="48" t="s">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="40" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="147" customHeight="1" spans="1:11">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="46" t="s">
+      <c r="E5" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="41" t="s">
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="36" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="164" customHeight="1" spans="1:11">
-      <c r="A6" s="26"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="22" t="s">
+      <c r="A6" s="15"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="46" t="s">
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="46" t="s">
+      <c r="I6" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="46" t="s">
+      <c r="J6" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="41" t="s">
+      <c r="K6" s="36" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="176.4" customHeight="1" spans="1:11">
-      <c r="A7" s="26"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="22" t="s">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="29"/>
-      <c r="G7" s="29"/>
-      <c r="H7" s="25" t="s">
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="41" t="s">
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="36" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="176.4" customHeight="1" spans="1:11">
-      <c r="A8" s="26"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="22" t="s">
+      <c r="A8" s="15"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="49" t="s">
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="I8" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="29"/>
-      <c r="K8" s="42" t="s">
+      <c r="J8" s="22"/>
+      <c r="K8" s="29" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="32" t="s">
+      <c r="D9" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="25" t="s">
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
-      <c r="K9" s="31" t="s">
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="32" t="s">
+      <c r="D10" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="25" t="s">
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
-      <c r="K10" s="31" t="s">
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="32" t="s">
+      <c r="D11" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="25" t="s">
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
-      <c r="K11" s="31" t="s">
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="32" t="s">
+      <c r="D12" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="25" t="s">
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="31" t="s">
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="32" t="s">
+      <c r="D13" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="25" t="s">
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-      <c r="K13" s="31" t="s">
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="21" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="32" t="s">
+      <c r="D14" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="25" t="s">
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="31" t="s">
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="D15" s="32" t="s">
+      <c r="D15" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="25" t="s">
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="31" t="s">
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="21" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="31" t="s">
+      <c r="E16" s="28" t="s">
         <v>71</v>
+      </c>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="31" t="s">
+      <c r="A17" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="B17" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="32" t="s">
+      <c r="C17" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="31" t="s">
-        <v>75</v>
+      <c r="E17" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="31" t="s">
+      <c r="A18" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="C18" s="31" t="s">
+      <c r="B18" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="D18" s="32" t="s">
+      <c r="C18" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E18" s="25" t="s">
+      <c r="D18" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25" t="s">
+      <c r="E18" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="43" t="s">
-        <v>81</v>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="37" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="33"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="44" t="s">
-        <v>83</v>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="38" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="33"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="E20" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25" t="s">
+      <c r="A20" s="23"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="44" t="s">
-        <v>85</v>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="38" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="21" ht="31" customHeight="1" spans="1:11">
-      <c r="A21" s="33"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="E21" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25" t="s">
+      <c r="A21" s="23"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="28"/>
-      <c r="J21" s="28"/>
-      <c r="K21" s="44" t="s">
-        <v>87</v>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="38" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="22" ht="62.4" spans="1:11">
-      <c r="A22" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="B22" s="20" t="s">
+      <c r="A22" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="B22" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="C22" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="E22" s="46" t="s">
+      <c r="D22" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="F22" s="46" t="s">
+      <c r="E22" s="39" t="s">
         <v>93</v>
       </c>
-      <c r="G22" s="46" t="s">
+      <c r="F22" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="H22" s="25" t="s">
+      <c r="G22" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="50" t="s">
+      <c r="H22" s="20" t="s">
         <v>96</v>
+      </c>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="42" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="23" ht="109.2" spans="1:11">
-      <c r="A23" s="34"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="22" t="s">
-        <v>97</v>
-      </c>
-      <c r="E23" s="25" t="s">
+      <c r="A23" s="29"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="I23" s="23" t="s">
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="J23" s="23" t="s">
+      <c r="I23" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="K23" s="45" t="s">
+      <c r="J23" s="19" t="s">
         <v>101</v>
+      </c>
+      <c r="K23" s="36" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="24" ht="172" customHeight="1" spans="1:11">
-      <c r="A24" s="34" t="s">
-        <v>102</v>
-      </c>
-      <c r="B24" s="27" t="s">
+      <c r="A24" s="29" t="s">
         <v>103</v>
       </c>
-      <c r="C24" s="27" t="s">
+      <c r="B24" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="C24" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="D24" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="E24" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="46" t="s">
-        <v>106</v>
-      </c>
-      <c r="I24" s="23" t="s">
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="J24" s="51" t="s">
+      <c r="I24" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="K24" s="45" t="s">
+      <c r="J24" s="43" t="s">
         <v>109</v>
+      </c>
+      <c r="K24" s="36" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="25" ht="163" customHeight="1" spans="1:11">
-      <c r="A25" s="34"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="E25" s="25" t="s">
+      <c r="A25" s="29"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="46" t="s">
-        <v>111</v>
-      </c>
-      <c r="I25" s="23" t="s">
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="J25" s="51" t="s">
+      <c r="I25" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="K25" s="45" t="s">
+      <c r="J25" s="43" t="s">
         <v>114</v>
+      </c>
+      <c r="K25" s="36" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="26" ht="126" customHeight="1" spans="1:11">
-      <c r="A26" s="35" t="s">
-        <v>115</v>
-      </c>
-      <c r="B26" s="35" t="s">
+      <c r="A26" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="C26" s="35" t="s">
+      <c r="B26" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="C26" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="52" t="s">
-        <v>118</v>
-      </c>
-      <c r="F26" s="23" t="s">
+      <c r="E26" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="F26" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="51" t="s">
-        <v>119</v>
-      </c>
-      <c r="H26" s="25" t="s">
+      <c r="G26" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="H26" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
-      <c r="K26" s="33" t="s">
-        <v>120</v>
+      <c r="I26" s="21"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="23" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="35" t="s">
-        <v>121</v>
-      </c>
-      <c r="B27" s="20" t="s">
+      <c r="A27" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="B27" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="22" t="s">
+      <c r="C27" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="25" t="s">
+      <c r="E27" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I27" s="28"/>
-      <c r="J27" s="28"/>
-      <c r="K27" s="48" t="s">
-        <v>125</v>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="40" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="28" ht="96" customHeight="1" spans="1:11">
-      <c r="A28" s="34" t="s">
-        <v>126</v>
-      </c>
-      <c r="B28" s="20" t="s">
+      <c r="A28" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="C28" s="20" t="s">
+      <c r="B28" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="C28" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="D28" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="53" t="s">
-        <v>129</v>
-      </c>
-      <c r="F28" s="23" t="s">
+      <c r="E28" s="45" t="s">
+        <v>130</v>
+      </c>
+      <c r="F28" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G28" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="H28" s="25" t="s">
+      <c r="G28" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="H28" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28"/>
-      <c r="K28" s="45" t="s">
-        <v>131</v>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="36" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="29" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A29" s="34"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="E29" s="25" t="s">
+      <c r="A29" s="29"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="E29" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="46" t="s">
-        <v>133</v>
-      </c>
-      <c r="I29" s="23" t="s">
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="39" t="s">
         <v>134</v>
       </c>
-      <c r="J29" s="46" t="s">
+      <c r="I29" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="K29" s="45" t="s">
+      <c r="J29" s="39" t="s">
         <v>136</v>
+      </c>
+      <c r="K29" s="36" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="35" t="s">
-        <v>137</v>
-      </c>
-      <c r="B30" s="20" t="s">
+      <c r="A30" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="B30" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="C30" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E30" s="25" t="s">
-        <v>140</v>
-      </c>
-      <c r="F30" s="28"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="25" t="s">
+      <c r="E30" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I30" s="28"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="20" t="s">
-        <v>141</v>
+      <c r="I30" s="21"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="16" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" ht="46.8" spans="1:11">
+      <c r="A31" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>145</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="E31" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31" s="33" t="s">
+        <v>148</v>
+      </c>
+      <c r="G31" s="33" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="16" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="64">
+  <mergeCells count="65">
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H4:J4"/>
@@ -2790,6 +2992,7 @@
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="E30:G30"/>
     <mergeCell ref="H30:J30"/>
+    <mergeCell ref="H31:J31"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A18:A21"/>
@@ -2814,5 +3017,6 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
version 20 - Added Admin right control to add new product
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="152">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -381,6 +381,20 @@
 }</t>
   </si>
   <si>
+    <t>// For testing purpose
+   res.status(200).send(
+   [{
+      "name" : `${req.body.productname}`,
+      "type" : `${req.body.producttype}`,
+      "group" : `${req.body.productgroup}`,
+      "brand" : `${req.body.productbrand}`,
+      "price" : `${req.body.productprice}`,
+      "price_range" : `${req.body.productpricerange}`,
+      "color" : `${req.body.productcolor}`,
+      "image" : `${req.body.productimage}`,
+   }]);</t>
+  </si>
+  <si>
     <t>CANDLES_AddNewProduct_URL</t>
   </si>
   <si>
@@ -623,12 +637,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Times New Roman"/>
-        <charset val="134"/>
-      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -640,7 +648,31 @@
       <t xml:space="preserve">
 [{
     "Currentuser" : `${req.session.personal_information.username}`,
-     "SessionID" : `${req.sessionID}`
+     "SessionID" : `${req.sessionID}`,
+     "isAdminRights" : false
+}]
++</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> If user is admin:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+[{
+    "Currentuser" : `${req.session.personal_information.username}`,
+     "SessionID" : `${req.sessionID}`,
+     "isAdminRights" : true
 }]
 </t>
     </r>
@@ -662,7 +694,8 @@
       </rPr>
       <t xml:space="preserve">[{
     "Currentuser" : undefined,
-    "SessionID" : undefined
+    "SessionID" : undefined,
+    "isAdminRights" : false
 }]
 </t>
     </r>
@@ -1180,6 +1213,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1187,12 +1226,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1652,7 +1685,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1718,22 +1751,25 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1751,17 +1787,17 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -1771,6 +1807,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
@@ -2169,7 +2208,7 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="35" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2196,7 +2235,7 @@
       <c r="J3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="35"/>
+      <c r="K3" s="36"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
       <c r="A4" s="15" t="s">
@@ -2211,13 +2250,13 @@
       <c r="D4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="40" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="40" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="20" t="s">
@@ -2225,7 +2264,7 @@
       </c>
       <c r="I4" s="21"/>
       <c r="J4" s="21"/>
-      <c r="K4" s="40" t="s">
+      <c r="K4" s="41" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2242,13 +2281,13 @@
       <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="40" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="40" t="s">
         <v>25</v>
       </c>
       <c r="H5" s="20" t="s">
@@ -2256,7 +2295,7 @@
       </c>
       <c r="I5" s="21"/>
       <c r="J5" s="21"/>
-      <c r="K5" s="36" t="s">
+      <c r="K5" s="37" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2272,16 +2311,16 @@
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
-      <c r="H6" s="39" t="s">
+      <c r="H6" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="I6" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="39" t="s">
+      <c r="J6" s="40" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="36" t="s">
+      <c r="K6" s="37" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2292,7 +2331,7 @@
       <c r="D7" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="42" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="22"/>
@@ -2302,11 +2341,11 @@
       </c>
       <c r="I7" s="21"/>
       <c r="J7" s="21"/>
-      <c r="K7" s="36" t="s">
+      <c r="K7" s="37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" s="1" customFormat="1" ht="176.4" customHeight="1" spans="1:11">
+    <row r="8" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
       <c r="A8" s="15"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2318,32 +2357,34 @@
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="41" t="s">
+      <c r="H8" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="22"/>
-      <c r="K8" s="29" t="s">
+      <c r="J8" s="23" t="s">
         <v>38</v>
+      </c>
+      <c r="K8" s="30" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="23" t="s">
-        <v>39</v>
+      <c r="A9" s="24" t="s">
+        <v>40</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
@@ -2353,24 +2394,24 @@
       <c r="I9" s="21"/>
       <c r="J9" s="21"/>
       <c r="K9" s="21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="23" t="s">
-        <v>44</v>
+      <c r="A10" s="24" t="s">
+        <v>45</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
@@ -2380,24 +2421,24 @@
       <c r="I10" s="21"/>
       <c r="J10" s="21"/>
       <c r="K10" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="23" t="s">
-        <v>48</v>
+      <c r="A11" s="24" t="s">
+        <v>49</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
@@ -2407,24 +2448,24 @@
       <c r="I11" s="21"/>
       <c r="J11" s="21"/>
       <c r="K11" s="21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="23" t="s">
-        <v>52</v>
+      <c r="A12" s="24" t="s">
+        <v>53</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F12" s="21"/>
       <c r="G12" s="21"/>
@@ -2434,24 +2475,24 @@
       <c r="I12" s="21"/>
       <c r="J12" s="21"/>
       <c r="K12" s="21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="23" t="s">
-        <v>56</v>
+      <c r="A13" s="24" t="s">
+        <v>57</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F13" s="21"/>
       <c r="G13" s="21"/>
@@ -2461,24 +2502,24 @@
       <c r="I13" s="21"/>
       <c r="J13" s="21"/>
       <c r="K13" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="23" t="s">
-        <v>60</v>
+      <c r="A14" s="24" t="s">
+        <v>61</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="D14" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="21"/>
@@ -2488,24 +2529,24 @@
       <c r="I14" s="21"/>
       <c r="J14" s="21"/>
       <c r="K14" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="23" t="s">
-        <v>64</v>
+      <c r="A15" s="24" t="s">
+        <v>65</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
@@ -2515,78 +2556,78 @@
       <c r="I15" s="21"/>
       <c r="J15" s="21"/>
       <c r="K15" s="21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="26" t="s">
+      <c r="A16" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="B16" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="C16" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="I16" s="26"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="26" t="s">
+      <c r="E16" s="29" t="s">
         <v>72</v>
+      </c>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B17" s="26" t="s">
+      <c r="A17" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="B17" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="C17" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-      <c r="H17" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="I17" s="26"/>
-      <c r="J17" s="26"/>
-      <c r="K17" s="26" t="s">
-        <v>76</v>
+      <c r="E17" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="23" t="s">
-        <v>77</v>
+      <c r="A18" s="24" t="s">
+        <v>78</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="D18" s="24" t="s">
         <v>80</v>
       </c>
+      <c r="D18" s="25" t="s">
+        <v>81</v>
+      </c>
       <c r="E18" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
@@ -2595,19 +2636,19 @@
       </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
-      <c r="K18" s="37" t="s">
-        <v>82</v>
+      <c r="K18" s="38" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="23"/>
+      <c r="A19" s="24"/>
       <c r="B19" s="21"/>
       <c r="C19" s="21"/>
-      <c r="D19" s="24" t="s">
-        <v>83</v>
+      <c r="D19" s="25" t="s">
+        <v>84</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
@@ -2616,19 +2657,19 @@
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
-      <c r="K19" s="38" t="s">
-        <v>84</v>
+      <c r="K19" s="39" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="23"/>
+      <c r="A20" s="24"/>
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>
-      <c r="D20" s="24" t="s">
-        <v>85</v>
+      <c r="D20" s="25" t="s">
+        <v>86</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
@@ -2637,19 +2678,19 @@
       </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
-      <c r="K20" s="38" t="s">
-        <v>86</v>
+      <c r="K20" s="39" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="21" ht="31" customHeight="1" spans="1:11">
-      <c r="A21" s="23"/>
+      <c r="A21" s="24"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
-      <c r="D21" s="24" t="s">
-        <v>87</v>
+      <c r="D21" s="25" t="s">
+        <v>88</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
@@ -2658,251 +2699,251 @@
       </c>
       <c r="I21" s="21"/>
       <c r="J21" s="21"/>
-      <c r="K21" s="38" t="s">
-        <v>88</v>
+      <c r="K21" s="39" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="22" ht="62.4" spans="1:11">
-      <c r="A22" s="29" t="s">
-        <v>89</v>
+      <c r="A22" s="30" t="s">
+        <v>90</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="E22" s="39" t="s">
         <v>93</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="E22" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="G22" s="39" t="s">
+      <c r="F22" s="40" t="s">
         <v>95</v>
       </c>
+      <c r="G22" s="40" t="s">
+        <v>96</v>
+      </c>
       <c r="H22" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I22" s="21"/>
       <c r="J22" s="21"/>
-      <c r="K22" s="42" t="s">
-        <v>97</v>
+      <c r="K22" s="44" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="23" ht="109.2" spans="1:11">
-      <c r="A23" s="29"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
       <c r="D23" s="18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E23" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="39" t="s">
-        <v>99</v>
+      <c r="H23" s="40" t="s">
+        <v>100</v>
       </c>
       <c r="I23" s="19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="K23" s="36" t="s">
         <v>102</v>
       </c>
+      <c r="K23" s="37" t="s">
+        <v>103</v>
+      </c>
     </row>
-    <row r="24" ht="172" customHeight="1" spans="1:11">
-      <c r="A24" s="29" t="s">
-        <v>103</v>
+    <row r="24" ht="314" customHeight="1" spans="1:11">
+      <c r="A24" s="30" t="s">
+        <v>104</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="39" t="s">
-        <v>107</v>
+      <c r="H24" s="40" t="s">
+        <v>108</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>108</v>
-      </c>
-      <c r="J24" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="K24" s="36" t="s">
+      <c r="J24" s="45" t="s">
         <v>110</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="25" ht="163" customHeight="1" spans="1:11">
-      <c r="A25" s="29"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
       <c r="D25" s="18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E25" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="39" t="s">
-        <v>112</v>
+      <c r="H25" s="40" t="s">
+        <v>113</v>
       </c>
       <c r="I25" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="J25" s="43" t="s">
         <v>114</v>
       </c>
-      <c r="K25" s="36" t="s">
+      <c r="J25" s="45" t="s">
         <v>115</v>
+      </c>
+      <c r="K25" s="37" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="26" ht="126" customHeight="1" spans="1:11">
-      <c r="A26" s="29" t="s">
-        <v>116</v>
-      </c>
-      <c r="B26" s="29" t="s">
+      <c r="A26" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="C26" s="29" t="s">
+      <c r="B26" s="30" t="s">
         <v>118</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>119</v>
       </c>
       <c r="D26" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="44" t="s">
-        <v>119</v>
+      <c r="E26" s="46" t="s">
+        <v>120</v>
       </c>
       <c r="F26" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="43" t="s">
-        <v>120</v>
+      <c r="G26" s="45" t="s">
+        <v>121</v>
       </c>
       <c r="H26" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I26" s="21"/>
       <c r="J26" s="21"/>
-      <c r="K26" s="23" t="s">
-        <v>121</v>
+      <c r="K26" s="24" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:11">
-      <c r="A27" s="29" t="s">
-        <v>122</v>
+      <c r="A27" s="30" t="s">
+        <v>123</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="28" t="s">
-        <v>125</v>
-      </c>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
+      <c r="E27" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
       <c r="H27" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="21"/>
-      <c r="K27" s="40" t="s">
-        <v>126</v>
+      <c r="K27" s="41" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="28" ht="96" customHeight="1" spans="1:11">
-      <c r="A28" s="29" t="s">
-        <v>127</v>
+      <c r="A28" s="30" t="s">
+        <v>128</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="45" t="s">
-        <v>130</v>
+      <c r="E28" s="47" t="s">
+        <v>131</v>
       </c>
       <c r="F28" s="19" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H28" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I28" s="21"/>
       <c r="J28" s="21"/>
-      <c r="K28" s="36" t="s">
-        <v>132</v>
+      <c r="K28" s="37" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="29" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A29" s="29"/>
+      <c r="A29" s="30"/>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="18" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E29" s="20" t="s">
         <v>19</v>
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="39" t="s">
-        <v>134</v>
+      <c r="H29" s="40" t="s">
+        <v>135</v>
       </c>
       <c r="I29" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="J29" s="39" t="s">
         <v>136</v>
       </c>
-      <c r="K29" s="36" t="s">
+      <c r="J29" s="40" t="s">
         <v>137</v>
+      </c>
+      <c r="K29" s="37" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="1:11">
-      <c r="A30" s="29" t="s">
-        <v>138</v>
+      <c r="A30" s="30" t="s">
+        <v>139</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C30" s="16" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D30" s="18" t="s">
         <v>15</v>
       </c>
       <c r="E30" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
@@ -2912,30 +2953,30 @@
       <c r="I30" s="21"/>
       <c r="J30" s="21"/>
       <c r="K30" s="16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" ht="46.8" spans="1:11">
-      <c r="A31" s="29" t="s">
-        <v>143</v>
+      <c r="A31" s="30" t="s">
+        <v>144</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="E31" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="F31" s="33" t="s">
+      <c r="E31" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="G31" s="33" t="s">
+      <c r="F31" s="34" t="s">
         <v>149</v>
+      </c>
+      <c r="G31" s="34" t="s">
+        <v>150</v>
       </c>
       <c r="H31" s="20" t="s">
         <v>19</v>
@@ -2943,7 +2984,7 @@
       <c r="I31" s="21"/>
       <c r="J31" s="21"/>
       <c r="K31" s="16" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version 25 - (Continue migration) Merge selected product in local storage with Redis and DB after login
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Server APIs'!$E$1:$G$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Server APIs'!$E$1:$G$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="156">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -637,6 +637,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -902,6 +908,21 @@
   </si>
   <si>
     <t>PAYMENT_HANDLING_Specific_Handling_URL</t>
+  </si>
+  <si>
+    <t>/mergelocalstorageandDB</t>
+  </si>
+  <si>
+    <t>- Get user information (sessionID in cookie is enough) and selected product from local storage before login
+- Merge data in local storage to data in Database
+- Delete old selected product data in Redis</t>
+  </si>
+  <si>
+    <t>Request header (included Cookie for authentication)
+Must content info personal_shopping_bag in UserInformation model (to read all data from local storage and send to Server)</t>
+  </si>
+  <si>
+    <t>PAYMENT_HANDLING_Merge_local_storage_and_DB</t>
   </si>
   <si>
     <t>API 18: Shopping bag handling</t>
@@ -1416,7 +1437,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1434,6 +1455,43 @@
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -1561,7 +1619,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1573,34 +1631,34 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1685,7 +1743,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1778,8 +1836,26 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2163,7 +2239,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
@@ -2208,7 +2284,7 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="35" t="s">
+      <c r="K2" s="41" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2235,7 +2311,7 @@
       <c r="J3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="36"/>
+      <c r="K3" s="42"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
       <c r="A4" s="15" t="s">
@@ -2250,13 +2326,13 @@
       <c r="D4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="46" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="40" t="s">
+      <c r="G4" s="46" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="20" t="s">
@@ -2264,7 +2340,7 @@
       </c>
       <c r="I4" s="21"/>
       <c r="J4" s="21"/>
-      <c r="K4" s="41" t="s">
+      <c r="K4" s="47" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2281,13 +2357,13 @@
       <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="46" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="40" t="s">
+      <c r="G5" s="46" t="s">
         <v>25</v>
       </c>
       <c r="H5" s="20" t="s">
@@ -2295,7 +2371,7 @@
       </c>
       <c r="I5" s="21"/>
       <c r="J5" s="21"/>
-      <c r="K5" s="37" t="s">
+      <c r="K5" s="43" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2311,16 +2387,16 @@
       </c>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="40" t="s">
+      <c r="I6" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="40" t="s">
+      <c r="J6" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="37" t="s">
+      <c r="K6" s="43" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2331,7 +2407,7 @@
       <c r="D7" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="42" t="s">
+      <c r="E7" s="48" t="s">
         <v>33</v>
       </c>
       <c r="F7" s="22"/>
@@ -2341,7 +2417,7 @@
       </c>
       <c r="I7" s="21"/>
       <c r="J7" s="21"/>
-      <c r="K7" s="37" t="s">
+      <c r="K7" s="43" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2357,7 +2433,7 @@
       </c>
       <c r="F8" s="21"/>
       <c r="G8" s="21"/>
-      <c r="H8" s="43" t="s">
+      <c r="H8" s="49" t="s">
         <v>36</v>
       </c>
       <c r="I8" s="23" t="s">
@@ -2636,7 +2712,7 @@
       </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21"/>
-      <c r="K18" s="38" t="s">
+      <c r="K18" s="44" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2657,7 +2733,7 @@
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
-      <c r="K19" s="39" t="s">
+      <c r="K19" s="45" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2678,7 +2754,7 @@
       </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
-      <c r="K20" s="39" t="s">
+      <c r="K20" s="45" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2699,7 +2775,7 @@
       </c>
       <c r="I21" s="21"/>
       <c r="J21" s="21"/>
-      <c r="K21" s="39" t="s">
+      <c r="K21" s="45" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2716,13 +2792,13 @@
       <c r="D22" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="40" t="s">
+      <c r="E22" s="46" t="s">
         <v>94</v>
       </c>
-      <c r="F22" s="40" t="s">
+      <c r="F22" s="46" t="s">
         <v>95</v>
       </c>
-      <c r="G22" s="40" t="s">
+      <c r="G22" s="46" t="s">
         <v>96</v>
       </c>
       <c r="H22" s="20" t="s">
@@ -2730,7 +2806,7 @@
       </c>
       <c r="I22" s="21"/>
       <c r="J22" s="21"/>
-      <c r="K22" s="44" t="s">
+      <c r="K22" s="50" t="s">
         <v>98</v>
       </c>
     </row>
@@ -2746,7 +2822,7 @@
       </c>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="46" t="s">
         <v>100</v>
       </c>
       <c r="I23" s="19" t="s">
@@ -2755,7 +2831,7 @@
       <c r="J23" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="K23" s="37" t="s">
+      <c r="K23" s="43" t="s">
         <v>103</v>
       </c>
     </row>
@@ -2777,16 +2853,16 @@
       </c>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="40" t="s">
+      <c r="H24" s="46" t="s">
         <v>108</v>
       </c>
       <c r="I24" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="J24" s="45" t="s">
+      <c r="J24" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="K24" s="37" t="s">
+      <c r="K24" s="43" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2802,16 +2878,16 @@
       </c>
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
-      <c r="H25" s="40" t="s">
+      <c r="H25" s="46" t="s">
         <v>113</v>
       </c>
       <c r="I25" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="J25" s="45" t="s">
+      <c r="J25" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="K25" s="37" t="s">
+      <c r="K25" s="43" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2828,13 +2904,13 @@
       <c r="D26" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="52" t="s">
         <v>120</v>
       </c>
       <c r="F26" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="45" t="s">
+      <c r="G26" s="51" t="s">
         <v>121</v>
       </c>
       <c r="H26" s="20" t="s">
@@ -2869,24 +2945,24 @@
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="21"/>
-      <c r="K27" s="41" t="s">
+      <c r="K27" s="47" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="28" ht="96" customHeight="1" spans="1:11">
-      <c r="A28" s="30" t="s">
+      <c r="A28" s="32" t="s">
         <v>128</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="33" t="s">
         <v>129</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="33" t="s">
         <v>130</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="47" t="s">
+      <c r="E28" s="53" t="s">
         <v>131</v>
       </c>
       <c r="F28" s="19" t="s">
@@ -2900,14 +2976,14 @@
       </c>
       <c r="I28" s="21"/>
       <c r="J28" s="21"/>
-      <c r="K28" s="37" t="s">
+      <c r="K28" s="43" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="29" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A29" s="30"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
+      <c r="A29" s="35"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
       <c r="D29" s="18" t="s">
         <v>134</v>
       </c>
@@ -2916,75 +2992,98 @@
       </c>
       <c r="F29" s="21"/>
       <c r="G29" s="21"/>
-      <c r="H29" s="40" t="s">
+      <c r="H29" s="46" t="s">
         <v>135</v>
       </c>
       <c r="I29" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="J29" s="40" t="s">
+      <c r="J29" s="46" t="s">
         <v>137</v>
       </c>
-      <c r="K29" s="37" t="s">
+      <c r="K29" s="43" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
-      <c r="A30" s="30" t="s">
+    <row r="30" ht="141" customHeight="1" spans="1:11">
+      <c r="A30" s="37"/>
+      <c r="B30" s="38"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="B30" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="D30" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E30" s="20" t="s">
-        <v>142</v>
-      </c>
+      <c r="E30" s="20"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
-      <c r="H30" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="16" t="s">
+      <c r="H30" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="I30" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="J30" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="K30" s="43" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31" s="30" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="31" ht="46.8" spans="1:11">
-      <c r="A31" s="30" t="s">
+      <c r="B31" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="C31" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="D31" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="D31" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" s="33" t="s">
-        <v>148</v>
-      </c>
-      <c r="F31" s="34" t="s">
-        <v>149</v>
-      </c>
-      <c r="G31" s="34" t="s">
-        <v>150</v>
-      </c>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
       <c r="H31" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I31" s="21"/>
       <c r="J31" s="21"/>
       <c r="K31" s="16" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" ht="46.8" spans="1:11">
+      <c r="A32" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="D32" s="18" t="s">
         <v>151</v>
+      </c>
+      <c r="E32" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="F32" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="16" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3031,27 +3130,27 @@
     <mergeCell ref="H27:J27"/>
     <mergeCell ref="H28:J28"/>
     <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="E31:G31"/>
     <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H32:J32"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A8"/>
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A28:A30"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B5:B8"/>
     <mergeCell ref="B18:B21"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="B28:B30"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="C5:C8"/>
     <mergeCell ref="C18:C21"/>
     <mergeCell ref="C22:C23"/>
     <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="C28:C30"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="K2:K3"/>
   </mergeCells>

</xml_diff>

<commit_message>
version 26 - (Completed migration) Add remove button for admin only to remove waste product
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Server APIs'!$E$1:$G$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Server APIs'!$E$1:$G$32</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +35,7 @@
     <author>PC</author>
   </authors>
   <commentList>
-    <comment ref="K16" authorId="0">
+    <comment ref="K17" authorId="0">
       <text>
         <r>
           <rPr>
@@ -57,7 +57,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K17" authorId="0">
+    <comment ref="K18" authorId="0">
       <text>
         <r>
           <rPr>
@@ -80,7 +80,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K18" authorId="0">
+    <comment ref="K19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -99,29 +99,6 @@
           </rPr>
           <t xml:space="preserve">
 Handle internal in Angular, dont contact to server now</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K19" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Times New Roman"/>
-            <charset val="0"/>
-          </rPr>
-          <t>PC:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Times New Roman"/>
-            <charset val="0"/>
-          </rPr>
-          <t xml:space="preserve">
-Handle internal in Angular, dont contact to server now
-</t>
         </r>
       </text>
     </comment>
@@ -171,12 +148,35 @@
         </r>
       </text>
     </comment>
+    <comment ref="K22" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>PC:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Handle internal in Angular, dont contact to server now
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="160">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -396,6 +396,30 @@
   </si>
   <si>
     <t>CANDLES_AddNewProduct_URL</t>
+  </si>
+  <si>
+    <t>/RemoveProduct</t>
+  </si>
+  <si>
+    <t>- Remove product into Database and Redis cache</t>
+  </si>
+  <si>
+    <t>// For testing purpose
+   res.status(200).send(
+   [{
+      "name" : `${req.body.productname}`,
+      "type" : `${req.body.producttype}`,
+      "group" : `${req.body.productgroup}`,
+      "brand" : `${req.body.productbrand}`,
+      "price" : `${req.body.productprice}`,
+      "price_range" : `${req.body.productpricerange}`,
+      "color" : `${req.body.productcolor}`,
+      "image" : `${req.body.productimage}`,
+      "status_of_removed_product" : "Remove product successfully/unsuccessfully"
+   }]);</t>
+  </si>
+  <si>
+    <t>CANDLES_By_RequestToBeRemoved</t>
   </si>
   <si>
     <t>API 3:  Oils product route</t>
@@ -2239,7 +2263,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
@@ -2446,48 +2470,44 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="24" t="s">
+    <row r="9" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
+      <c r="A9" s="15"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>43</v>
-      </c>
+      <c r="E9" s="20"/>
       <c r="F9" s="21"/>
       <c r="G9" s="21"/>
-      <c r="H9" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="21"/>
-      <c r="J9" s="21"/>
-      <c r="K9" s="21" t="s">
-        <v>44</v>
+      <c r="H9" s="49" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="C10" s="21" t="s">
         <v>46</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>47</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F10" s="21"/>
       <c r="G10" s="21"/>
@@ -2514,7 +2534,7 @@
         <v>15</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F11" s="21"/>
       <c r="G11" s="21"/>
@@ -2541,7 +2561,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F12" s="21"/>
       <c r="G12" s="21"/>
@@ -2568,7 +2588,7 @@
         <v>15</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F13" s="21"/>
       <c r="G13" s="21"/>
@@ -2595,7 +2615,7 @@
         <v>15</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F14" s="21"/>
       <c r="G14" s="21"/>
@@ -2622,7 +2642,7 @@
         <v>15</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F15" s="21"/>
       <c r="G15" s="21"/>
@@ -2636,52 +2656,52 @@
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="29" t="s">
+      <c r="E16" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" s="21"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="21" t="s">
         <v>72</v>
-      </c>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="29" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="27" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="C17" s="27" t="s">
         <v>75</v>
-      </c>
-      <c r="C17" s="27" t="s">
-        <v>76</v>
       </c>
       <c r="D17" s="28" t="s">
         <v>15</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F17" s="27"/>
       <c r="G17" s="27"/>
       <c r="H17" s="29" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="I17" s="27"/>
       <c r="J17" s="27"/>
@@ -2690,41 +2710,47 @@
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="24" t="s">
+      <c r="A18" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27" t="s">
         <v>81</v>
-      </c>
-      <c r="E18" s="20" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="44" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="24"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
+      <c r="A19" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>84</v>
+      </c>
       <c r="D19" s="25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
@@ -2733,8 +2759,8 @@
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21"/>
-      <c r="K19" s="45" t="s">
-        <v>85</v>
+      <c r="K19" s="44" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2742,10 +2768,10 @@
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>
       <c r="D20" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="E20" s="20" t="s">
         <v>86</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>82</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
@@ -2755,18 +2781,18 @@
       <c r="I20" s="21"/>
       <c r="J20" s="21"/>
       <c r="K20" s="45" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
-    <row r="21" ht="31" customHeight="1" spans="1:11">
+    <row r="21" spans="1:11">
       <c r="A21" s="24"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
       <c r="D21" s="25" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
@@ -2776,77 +2802,67 @@
       <c r="I21" s="21"/>
       <c r="J21" s="21"/>
       <c r="K21" s="45" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
-    <row r="22" ht="62.4" spans="1:11">
-      <c r="A22" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="C22" s="16" t="s">
+    <row r="22" ht="31" customHeight="1" spans="1:11">
+      <c r="A22" s="24"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="E22" s="46" t="s">
-        <v>94</v>
-      </c>
-      <c r="F22" s="46" t="s">
-        <v>95</v>
-      </c>
-      <c r="G22" s="46" t="s">
-        <v>96</v>
-      </c>
+      <c r="E22" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
       <c r="H22" s="20" t="s">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="I22" s="21"/>
       <c r="J22" s="21"/>
-      <c r="K22" s="50" t="s">
+      <c r="K22" s="45" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" ht="62.4" spans="1:11">
+      <c r="A23" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="46" t="s">
         <v>98</v>
       </c>
+      <c r="F23" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="H23" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="50" t="s">
+        <v>102</v>
+      </c>
     </row>
-    <row r="23" ht="109.2" spans="1:11">
-      <c r="A23" s="30"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="46" t="s">
-        <v>100</v>
-      </c>
-      <c r="I23" s="19" t="s">
-        <v>101</v>
-      </c>
-      <c r="J23" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="K23" s="43" t="s">
+    <row r="24" ht="109.2" spans="1:11">
+      <c r="A24" s="30"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="18" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="24" ht="314" customHeight="1" spans="1:11">
-      <c r="A24" s="30" t="s">
-        <v>104</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>106</v>
-      </c>
-      <c r="D24" s="18" t="s">
-        <v>107</v>
       </c>
       <c r="E24" s="20" t="s">
         <v>19</v>
@@ -2854,24 +2870,30 @@
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
       <c r="H24" s="46" t="s">
+        <v>104</v>
+      </c>
+      <c r="I24" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="J24" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="K24" s="43" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" ht="314" customHeight="1" spans="1:11">
+      <c r="A25" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="B25" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="J24" s="51" t="s">
+      <c r="C25" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="K24" s="43" t="s">
+      <c r="D25" s="18" t="s">
         <v>111</v>
-      </c>
-    </row>
-    <row r="25" ht="163" customHeight="1" spans="1:11">
-      <c r="A25" s="30"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="18" t="s">
-        <v>112</v>
       </c>
       <c r="E25" s="20" t="s">
         <v>19</v>
@@ -2879,211 +2901,236 @@
       <c r="F25" s="21"/>
       <c r="G25" s="21"/>
       <c r="H25" s="46" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="I25" s="19" t="s">
+      <c r="J25" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="J25" s="51" t="s">
+      <c r="K25" s="43" t="s">
         <v>115</v>
       </c>
-      <c r="K25" s="43" t="s">
+    </row>
+    <row r="26" ht="163" customHeight="1" spans="1:11">
+      <c r="A26" s="30"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="18" t="s">
         <v>116</v>
       </c>
+      <c r="E26" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="46" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="J26" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="K26" s="43" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="26" ht="126" customHeight="1" spans="1:11">
-      <c r="A26" s="30" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" s="30" t="s">
-        <v>118</v>
-      </c>
-      <c r="C26" s="30" t="s">
-        <v>119</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="52" t="s">
-        <v>120</v>
-      </c>
-      <c r="F26" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G26" s="51" t="s">
+    <row r="27" ht="126" customHeight="1" spans="1:11">
+      <c r="A27" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="H26" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="24" t="s">
+      <c r="B27" s="30" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27" s="30" t="s">
+      <c r="C27" s="30" t="s">
         <v>123</v>
-      </c>
-      <c r="B27" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="C27" s="16" t="s">
-        <v>125</v>
       </c>
       <c r="D27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
+      <c r="E27" s="52" t="s">
+        <v>124</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>125</v>
+      </c>
       <c r="H27" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="21"/>
-      <c r="K27" s="47" t="s">
+      <c r="K27" s="24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11">
+      <c r="A28" s="30" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="28" ht="96" customHeight="1" spans="1:11">
-      <c r="A28" s="32" t="s">
+      <c r="B28" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="B28" s="33" t="s">
+      <c r="C28" s="16" t="s">
         <v>129</v>
-      </c>
-      <c r="C28" s="33" t="s">
-        <v>130</v>
       </c>
       <c r="D28" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="53" t="s">
-        <v>131</v>
-      </c>
-      <c r="F28" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" s="19" t="s">
-        <v>132</v>
-      </c>
+      <c r="E28" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
       <c r="H28" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I28" s="21"/>
       <c r="J28" s="21"/>
-      <c r="K28" s="43" t="s">
+      <c r="K28" s="47" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="29" ht="96" customHeight="1" spans="1:11">
+      <c r="A29" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="33" t="s">
         <v>133</v>
       </c>
+      <c r="C29" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="53" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="H29" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I29" s="21"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="43" t="s">
+        <v>137</v>
+      </c>
     </row>
-    <row r="29" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A29" s="35"/>
-      <c r="B29" s="36"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="E29" s="20" t="s">
+    <row r="30" ht="258.6" customHeight="1" spans="1:11">
+      <c r="A30" s="35"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="E30" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
-      <c r="H29" s="46" t="s">
-        <v>135</v>
-      </c>
-      <c r="I29" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="J29" s="46" t="s">
-        <v>137</v>
-      </c>
-      <c r="K29" s="43" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="30" ht="141" customHeight="1" spans="1:11">
-      <c r="A30" s="37"/>
-      <c r="B30" s="38"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="18" t="s">
-        <v>139</v>
-      </c>
-      <c r="E30" s="20"/>
       <c r="F30" s="21"/>
       <c r="G30" s="21"/>
       <c r="H30" s="46" t="s">
+        <v>139</v>
+      </c>
+      <c r="I30" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="I30" s="19" t="s">
+      <c r="J30" s="46" t="s">
         <v>141</v>
-      </c>
-      <c r="J30" s="19" t="s">
-        <v>132</v>
       </c>
       <c r="K30" s="43" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
-      <c r="A31" s="30" t="s">
+    <row r="31" ht="141" customHeight="1" spans="1:11">
+      <c r="A31" s="37"/>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="18" t="s">
         <v>143</v>
       </c>
-      <c r="B31" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E31" s="20" t="s">
-        <v>146</v>
-      </c>
+      <c r="E31" s="20"/>
       <c r="F31" s="21"/>
       <c r="G31" s="21"/>
-      <c r="H31" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="I31" s="21"/>
-      <c r="J31" s="21"/>
-      <c r="K31" s="16" t="s">
+      <c r="H31" s="46" t="s">
+        <v>144</v>
+      </c>
+      <c r="I31" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="J31" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="K31" s="43" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" s="30" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="32" ht="46.8" spans="1:11">
-      <c r="A32" s="30" t="s">
+      <c r="B32" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="B32" s="16" t="s">
+      <c r="C32" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="D32" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="D32" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>152</v>
-      </c>
-      <c r="F32" s="40" t="s">
-        <v>153</v>
-      </c>
-      <c r="G32" s="40" t="s">
-        <v>154</v>
-      </c>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
       <c r="H32" s="20" t="s">
         <v>19</v>
       </c>
       <c r="I32" s="21"/>
       <c r="J32" s="21"/>
       <c r="K32" s="16" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="33" ht="46.8" spans="1:11">
+      <c r="A33" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="D33" s="18" t="s">
         <v>155</v>
+      </c>
+      <c r="E33" s="39" t="s">
+        <v>156</v>
+      </c>
+      <c r="F33" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="G33" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="H33" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="16" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -3095,8 +3142,6 @@
     <mergeCell ref="E6:G6"/>
     <mergeCell ref="H7:J7"/>
     <mergeCell ref="E8:G8"/>
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="H9:J9"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="E11:G11"/>
@@ -3121,36 +3166,38 @@
     <mergeCell ref="H20:J20"/>
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="H21:J21"/>
+    <mergeCell ref="E22:G22"/>
     <mergeCell ref="H22:J22"/>
-    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="E24:G24"/>
     <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E26:G26"/>
     <mergeCell ref="H27:J27"/>
+    <mergeCell ref="E28:G28"/>
     <mergeCell ref="H28:J28"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="E32:G32"/>
     <mergeCell ref="H32:J32"/>
+    <mergeCell ref="H33:J33"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A8"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A29:A31"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B5:B8"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B29:B31"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="C5:C8"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="C29:C31"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="K2:K3"/>
   </mergeCells>

</xml_diff>

<commit_message>
version 29 - Update Redis info in environment setting
</commit_message>
<xml_diff>
--- a/RESTFul_API.xlsx
+++ b/RESTFul_API.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8280"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Server APIs" sheetId="3" r:id="rId1"/>
@@ -1767,7 +1767,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1827,6 +1827,18 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1835,6 +1847,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2308,7 +2326,7 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="41" t="s">
+      <c r="K2" s="47" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2335,7 +2353,7 @@
       <c r="J3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="42"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
       <c r="A4" s="15" t="s">
@@ -2350,403 +2368,403 @@
       <c r="D4" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="52" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="46" t="s">
+      <c r="G4" s="52" t="s">
         <v>18</v>
       </c>
       <c r="H4" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="21"/>
-      <c r="J4" s="21"/>
-      <c r="K4" s="47" t="s">
+      <c r="I4" s="25"/>
+      <c r="J4" s="25"/>
+      <c r="K4" s="53" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="147" customHeight="1" spans="1:11">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="46" t="s">
+      <c r="E5" s="52" t="s">
         <v>24</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="46" t="s">
+      <c r="G5" s="52" t="s">
         <v>25</v>
       </c>
       <c r="H5" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="43" t="s">
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="49" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="164" customHeight="1" spans="1:11">
-      <c r="A6" s="15"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
+      <c r="A6" s="23"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="18" t="s">
         <v>27</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="46" t="s">
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="46" t="s">
+      <c r="I6" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="46" t="s">
+      <c r="J6" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="43" t="s">
+      <c r="K6" s="49" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="176.4" customHeight="1" spans="1:11">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
       <c r="H7" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21"/>
-      <c r="K7" s="43" t="s">
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="49" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
+      <c r="A8" s="23"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
       <c r="D8" s="18" t="s">
         <v>35</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="49" t="s">
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="23" t="s">
+      <c r="J8" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="K8" s="30" t="s">
+      <c r="K8" s="36" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
-      <c r="A9" s="15"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
       <c r="D9" s="18" t="s">
         <v>40</v>
       </c>
       <c r="E9" s="20"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="49" t="s">
+      <c r="F9" s="25"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="23" t="s">
+      <c r="J9" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="K9" s="30" t="s">
+      <c r="K9" s="36" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
       <c r="H10" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21" t="s">
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="25"/>
       <c r="H11" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21" t="s">
+      <c r="I11" s="25"/>
+      <c r="J11" s="25"/>
+      <c r="K11" s="25" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="25"/>
       <c r="H12" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21" t="s">
+      <c r="I12" s="25"/>
+      <c r="J12" s="25"/>
+      <c r="K12" s="25" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="C13" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="25" t="s">
+      <c r="D13" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E13" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
+      <c r="F13" s="25"/>
+      <c r="G13" s="25"/>
       <c r="H13" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21" t="s">
+      <c r="I13" s="25"/>
+      <c r="J13" s="25"/>
+      <c r="K13" s="25" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="30" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="D14" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
       <c r="H14" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="21"/>
-      <c r="J14" s="21"/>
-      <c r="K14" s="21" t="s">
+      <c r="I14" s="25"/>
+      <c r="J14" s="25"/>
+      <c r="K14" s="25" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="24" t="s">
+      <c r="A15" s="30" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E15" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
       <c r="H15" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21" t="s">
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="30" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="31" t="s">
         <v>15</v>
       </c>
       <c r="E16" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
       <c r="H16" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21" t="s">
+      <c r="I16" s="25"/>
+      <c r="J16" s="25"/>
+      <c r="K16" s="25" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="26" t="s">
+      <c r="A17" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="27" t="s">
+      <c r="C17" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="28" t="s">
+      <c r="D17" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="29" t="s">
+      <c r="E17" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="29" t="s">
+      <c r="F17" s="33"/>
+      <c r="G17" s="33"/>
+      <c r="H17" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="27" t="s">
+      <c r="I17" s="33"/>
+      <c r="J17" s="33"/>
+      <c r="K17" s="33" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="26" t="s">
+      <c r="A18" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="29" t="s">
+      <c r="F18" s="33"/>
+      <c r="G18" s="33"/>
+      <c r="H18" s="35" t="s">
         <v>76</v>
       </c>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="27" t="s">
+      <c r="I18" s="33"/>
+      <c r="J18" s="33"/>
+      <c r="K18" s="33" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="D19" s="31" t="s">
         <v>85</v>
       </c>
       <c r="E19" s="20" t="s">
@@ -2757,17 +2775,17 @@
       <c r="H19" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="44" t="s">
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="50" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="24"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="25" t="s">
+      <c r="A20" s="30"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="31" t="s">
         <v>88</v>
       </c>
       <c r="E20" s="20" t="s">
@@ -2778,17 +2796,17 @@
       <c r="H20" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="45" t="s">
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="51" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="24"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="25" t="s">
+      <c r="A21" s="30"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="31" t="s">
         <v>90</v>
       </c>
       <c r="E21" s="20" t="s">
@@ -2799,17 +2817,17 @@
       <c r="H21" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="45" t="s">
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="51" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="22" ht="31" customHeight="1" spans="1:11">
-      <c r="A22" s="24"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="25" t="s">
+      <c r="A22" s="30"/>
+      <c r="B22" s="25"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="31" t="s">
         <v>92</v>
       </c>
       <c r="E22" s="20" t="s">
@@ -2820,14 +2838,14 @@
       <c r="H22" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="45" t="s">
+      <c r="I22" s="25"/>
+      <c r="J22" s="25"/>
+      <c r="K22" s="51" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="23" ht="62.4" spans="1:11">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="36" t="s">
         <v>94</v>
       </c>
       <c r="B23" s="16" t="s">
@@ -2839,26 +2857,26 @@
       <c r="D23" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="52" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="46" t="s">
+      <c r="F23" s="52" t="s">
         <v>99</v>
       </c>
-      <c r="G23" s="46" t="s">
+      <c r="G23" s="52" t="s">
         <v>100</v>
       </c>
       <c r="H23" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="50" t="s">
+      <c r="I23" s="25"/>
+      <c r="J23" s="25"/>
+      <c r="K23" s="56" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="24" ht="109.2" spans="1:11">
-      <c r="A24" s="30"/>
+      <c r="A24" s="36"/>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="18" t="s">
@@ -2867,9 +2885,9 @@
       <c r="E24" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="46" t="s">
+      <c r="F24" s="25"/>
+      <c r="G24" s="25"/>
+      <c r="H24" s="52" t="s">
         <v>104</v>
       </c>
       <c r="I24" s="19" t="s">
@@ -2878,12 +2896,12 @@
       <c r="J24" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="K24" s="43" t="s">
+      <c r="K24" s="49" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="25" ht="314" customHeight="1" spans="1:11">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="36" t="s">
         <v>108</v>
       </c>
       <c r="B25" s="16" t="s">
@@ -2898,23 +2916,23 @@
       <c r="E25" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="46" t="s">
+      <c r="F25" s="25"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="52" t="s">
         <v>112</v>
       </c>
       <c r="I25" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="51" t="s">
+      <c r="J25" s="57" t="s">
         <v>114</v>
       </c>
-      <c r="K25" s="43" t="s">
+      <c r="K25" s="49" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="26" ht="163" customHeight="1" spans="1:11">
-      <c r="A26" s="30"/>
+      <c r="A26" s="36"/>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="18" t="s">
@@ -2923,54 +2941,54 @@
       <c r="E26" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="46" t="s">
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="52" t="s">
         <v>117</v>
       </c>
       <c r="I26" s="19" t="s">
         <v>118</v>
       </c>
-      <c r="J26" s="51" t="s">
+      <c r="J26" s="57" t="s">
         <v>119</v>
       </c>
-      <c r="K26" s="43" t="s">
+      <c r="K26" s="49" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="27" ht="126" customHeight="1" spans="1:11">
-      <c r="A27" s="30" t="s">
+      <c r="A27" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="B27" s="30" t="s">
+      <c r="B27" s="36" t="s">
         <v>122</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="36" t="s">
         <v>123</v>
       </c>
       <c r="D27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="52" t="s">
+      <c r="E27" s="58" t="s">
         <v>124</v>
       </c>
       <c r="F27" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="51" t="s">
+      <c r="G27" s="57" t="s">
         <v>125</v>
       </c>
       <c r="H27" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="24" t="s">
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="30" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="30" t="s">
+      <c r="A28" s="36" t="s">
         <v>127</v>
       </c>
       <c r="B28" s="16" t="s">
@@ -2982,34 +3000,34 @@
       <c r="D28" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="29" t="s">
+      <c r="E28" s="35" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
       <c r="H28" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I28" s="21"/>
-      <c r="J28" s="21"/>
-      <c r="K28" s="47" t="s">
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="53" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="29" ht="96" customHeight="1" spans="1:11">
-      <c r="A29" s="32" t="s">
+      <c r="A29" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="33" t="s">
+      <c r="B29" s="39" t="s">
         <v>133</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="39" t="s">
         <v>134</v>
       </c>
       <c r="D29" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="53" t="s">
+      <c r="E29" s="59" t="s">
         <v>135</v>
       </c>
       <c r="F29" s="19" t="s">
@@ -3021,48 +3039,48 @@
       <c r="H29" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I29" s="21"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="43" t="s">
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="49" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="30" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A30" s="35"/>
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
+      <c r="A30" s="41"/>
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
       <c r="D30" s="18" t="s">
         <v>138</v>
       </c>
       <c r="E30" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="46" t="s">
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="52" t="s">
         <v>139</v>
       </c>
       <c r="I30" s="19" t="s">
         <v>140</v>
       </c>
-      <c r="J30" s="46" t="s">
+      <c r="J30" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="K30" s="43" t="s">
+      <c r="K30" s="49" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="31" ht="141" customHeight="1" spans="1:11">
-      <c r="A31" s="37"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
+      <c r="A31" s="43"/>
+      <c r="B31" s="44"/>
+      <c r="C31" s="44"/>
       <c r="D31" s="18" t="s">
         <v>143</v>
       </c>
       <c r="E31" s="20"/>
-      <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
-      <c r="H31" s="46" t="s">
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="52" t="s">
         <v>144</v>
       </c>
       <c r="I31" s="19" t="s">
@@ -3071,12 +3089,12 @@
       <c r="J31" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="K31" s="43" t="s">
+      <c r="K31" s="49" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:11">
-      <c r="A32" s="30" t="s">
+      <c r="A32" s="36" t="s">
         <v>147</v>
       </c>
       <c r="B32" s="16" t="s">
@@ -3091,19 +3109,19 @@
       <c r="E32" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
       <c r="H32" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
       <c r="K32" s="16" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="33" ht="46.8" spans="1:11">
-      <c r="A33" s="30" t="s">
+      <c r="A33" s="36" t="s">
         <v>152</v>
       </c>
       <c r="B33" s="16" t="s">
@@ -3115,20 +3133,20 @@
       <c r="D33" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="E33" s="39" t="s">
+      <c r="E33" s="45" t="s">
         <v>156</v>
       </c>
-      <c r="F33" s="40" t="s">
+      <c r="F33" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="G33" s="40" t="s">
+      <c r="G33" s="46" t="s">
         <v>158</v>
       </c>
       <c r="H33" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="21"/>
-      <c r="J33" s="21"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
       <c r="K33" s="16" t="s">
         <v>159</v>
       </c>
@@ -3181,19 +3199,19 @@
     <mergeCell ref="H32:J32"/>
     <mergeCell ref="H33:J33"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="A5:A9"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A29:A31"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="B5:B9"/>
     <mergeCell ref="B19:B22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="B29:B31"/>
     <mergeCell ref="C2:C3"/>
-    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="C5:C9"/>
     <mergeCell ref="C19:C22"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="C25:C26"/>

</xml_diff>